<commit_message>
Relatório de OS para todas as OS's
</commit_message>
<xml_diff>
--- a/Relatorio_OS.xlsx
+++ b/Relatorio_OS.xlsx
@@ -953,7 +953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.85546875" customWidth="1" min="1" max="1"/>
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>1068</v>
+        <v>20</v>
       </c>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="7" t="n"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>18/03/2024</t>
+          <t>27/06/2023</t>
         </is>
       </c>
       <c r="H8" s="11" t="n"/>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="H9" s="11" t="n"/>
@@ -1111,11 +1111,7 @@
           <t>Solicitante:</t>
         </is>
       </c>
-      <c r="B10" s="57" t="inlineStr">
-        <is>
-          <t>004322 - FRANCISCO ALEX SOUSA FERREIRA</t>
-        </is>
-      </c>
+      <c r="B10" s="57" t="n"/>
       <c r="C10" s="58" t="n"/>
       <c r="D10" s="58" t="n"/>
       <c r="E10" s="59" t="n"/>
@@ -1165,7 +1161,7 @@
       </c>
       <c r="B12" s="51" t="inlineStr">
         <is>
-          <t>PRoblema na geração do laser</t>
+          <t>Problema na troca de mesa</t>
         </is>
       </c>
       <c r="C12" s="24" t="n"/>
@@ -1359,161 +1355,95 @@
       </c>
       <c r="B24" s="60" t="inlineStr">
         <is>
-          <t>O laser parou de ser gerado, sendo necessário enviar o módulo gerador para a autorizada omnitek</t>
+          <t>Regulagem do sensor da mesa</t>
         </is>
       </c>
       <c r="C24" s="61" t="n"/>
       <c r="D24" s="60" t="inlineStr">
         <is>
-          <t>004256,004389</t>
+          <t>{"[\"4363 - Davi\"]"}</t>
         </is>
       </c>
       <c r="E24" s="50" t="inlineStr">
         <is>
-          <t>06/12/2023</t>
+          <t>26/06/2023</t>
         </is>
       </c>
       <c r="F24" s="53" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6111111111111112</v>
       </c>
       <c r="G24" s="50" t="inlineStr">
         <is>
-          <t>08/12/2023</t>
+          <t>26/06/2023</t>
         </is>
       </c>
       <c r="H24" s="53" t="n">
-        <v>0.625</v>
+        <v>0.6180555555555556</v>
       </c>
     </row>
     <row r="25" ht="69" customHeight="1">
-      <c r="A25" s="60" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="60" t="inlineStr">
-        <is>
-          <t>Realizar a instalação do novo gerador e chiller</t>
-        </is>
-      </c>
+      <c r="A25" s="60" t="n"/>
+      <c r="B25" s="60" t="n"/>
       <c r="C25" s="61" t="n"/>
-      <c r="D25" s="60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E25" s="50" t="inlineStr">
-        <is>
-          <t>12/03/2024</t>
-        </is>
-      </c>
-      <c r="F25" s="53" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="G25" s="50" t="inlineStr">
-        <is>
-          <t>12/03/2024</t>
-        </is>
-      </c>
-      <c r="H25" s="53" t="n">
-        <v>0.9166666666666666</v>
-      </c>
-    </row>
-    <row r="26" ht="69" customHeight="1">
-      <c r="A26" s="60" t="n">
-        <v>3</v>
-      </c>
-      <c r="B26" s="60" t="inlineStr">
-        <is>
-          <t>Realizar testes e ajustes na máquina</t>
-        </is>
-      </c>
-      <c r="C26" s="61" t="n"/>
-      <c r="D26" s="60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E26" s="50" t="inlineStr">
-        <is>
-          <t>12/03/2024</t>
-        </is>
-      </c>
-      <c r="F26" s="53" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="G26" s="50" t="inlineStr">
-        <is>
-          <t>12/03/2024</t>
-        </is>
-      </c>
-      <c r="H26" s="53" t="n">
-        <v>0.7916666666666666</v>
-      </c>
-    </row>
-    <row r="27" ht="69" customHeight="1">
-      <c r="A27" s="60" t="n">
-        <v>4</v>
-      </c>
-      <c r="B27" s="60" t="inlineStr">
-        <is>
-          <t>Finalizar ajustes na máquina</t>
-        </is>
-      </c>
-      <c r="C27" s="61" t="n"/>
-      <c r="D27" s="60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E27" s="50" t="inlineStr">
-        <is>
-          <t>14/03/2024</t>
-        </is>
-      </c>
-      <c r="F27" s="53" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="G27" s="50" t="inlineStr">
-        <is>
-          <t>14/03/2024</t>
-        </is>
-      </c>
-      <c r="H27" s="53" t="n">
-        <v>0.7083333333333334</v>
-      </c>
-    </row>
-    <row r="28" ht="69" customHeight="1">
-      <c r="A28" s="60" t="n"/>
-      <c r="B28" s="60" t="n"/>
-      <c r="C28" s="61" t="n"/>
-      <c r="D28" s="60" t="n"/>
-      <c r="E28" s="50" t="n"/>
-      <c r="F28" s="50" t="n"/>
-      <c r="G28" s="50" t="n"/>
-      <c r="H28" s="50" t="n"/>
+      <c r="D25" s="60" t="n"/>
+      <c r="E25" s="50" t="n"/>
+      <c r="F25" s="50" t="n"/>
+      <c r="G25" s="50" t="n"/>
+      <c r="H25" s="50" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="n"/>
+      <c r="B27" s="73" t="n"/>
+      <c r="C27" s="68" t="n"/>
+      <c r="D27" s="41" t="n"/>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="41" t="n"/>
+      <c r="G27" s="41" t="n"/>
+      <c r="H27" s="41" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="37" t="n"/>
+      <c r="B28" s="38" t="n"/>
+      <c r="C28" s="38" t="n"/>
+      <c r="D28" s="39" t="inlineStr">
+        <is>
+          <t>Descrição do serviço</t>
+        </is>
+      </c>
+      <c r="E28" s="38" t="n"/>
+      <c r="F28" s="38" t="n"/>
+      <c r="G28" s="38" t="n"/>
+      <c r="H28" s="40" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="43" t="n"/>
+      <c r="B29" s="37" t="n"/>
+      <c r="C29" s="38" t="n"/>
+      <c r="D29" s="38" t="n"/>
+      <c r="E29" s="38" t="n"/>
+      <c r="F29" s="40" t="n"/>
+      <c r="G29" s="43" t="n"/>
+      <c r="H29" s="43" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="41" t="n"/>
-      <c r="B30" s="73" t="n"/>
-      <c r="C30" s="68" t="n"/>
-      <c r="D30" s="41" t="n"/>
-      <c r="E30" s="41" t="n"/>
-      <c r="F30" s="41" t="n"/>
-      <c r="G30" s="41" t="n"/>
-      <c r="H30" s="41" t="n"/>
+      <c r="A30" s="43" t="n"/>
+      <c r="B30" s="37" t="n"/>
+      <c r="C30" s="38" t="n"/>
+      <c r="D30" s="38" t="n"/>
+      <c r="E30" s="38" t="n"/>
+      <c r="F30" s="40" t="n"/>
+      <c r="G30" s="43" t="n"/>
+      <c r="H30" s="43" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="38" t="n"/>
+      <c r="A31" s="43" t="n"/>
+      <c r="B31" s="37" t="n"/>
       <c r="C31" s="38" t="n"/>
-      <c r="D31" s="39" t="inlineStr">
-        <is>
-          <t>Descrição do serviço</t>
-        </is>
-      </c>
+      <c r="D31" s="38" t="n"/>
       <c r="E31" s="38" t="n"/>
-      <c r="F31" s="38" t="n"/>
-      <c r="G31" s="38" t="n"/>
-      <c r="H31" s="40" t="n"/>
+      <c r="F31" s="40" t="n"/>
+      <c r="G31" s="43" t="n"/>
+      <c r="H31" s="43" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="43" t="n"/>
@@ -1526,24 +1456,37 @@
       <c r="H32" s="43" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="43" t="n"/>
-      <c r="B33" s="37" t="n"/>
-      <c r="C33" s="38" t="n"/>
-      <c r="D33" s="38" t="n"/>
-      <c r="E33" s="38" t="n"/>
-      <c r="F33" s="40" t="n"/>
-      <c r="G33" s="43" t="n"/>
-      <c r="H33" s="43" t="n"/>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>Materiais Utilizados</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="43" t="n"/>
-      <c r="B34" s="37" t="n"/>
-      <c r="C34" s="38" t="n"/>
-      <c r="D34" s="38" t="n"/>
-      <c r="E34" s="38" t="n"/>
-      <c r="F34" s="40" t="n"/>
-      <c r="G34" s="43" t="n"/>
-      <c r="H34" s="43" t="n"/>
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="B34" s="76" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n"/>
+      <c r="D34" s="58" t="n"/>
+      <c r="E34" s="58" t="n"/>
+      <c r="F34" s="58" t="n"/>
+      <c r="G34" s="48" t="inlineStr">
+        <is>
+          <t>Almox Retirada</t>
+        </is>
+      </c>
+      <c r="H34" s="48" t="inlineStr">
+        <is>
+          <t>Qtd</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="43" t="n"/>
@@ -1556,37 +1499,24 @@
       <c r="H35" s="43" t="n"/>
     </row>
     <row r="36">
-      <c r="D36" s="42" t="inlineStr">
-        <is>
-          <t>Materiais Utilizados</t>
-        </is>
-      </c>
+      <c r="A36" s="43" t="n"/>
+      <c r="B36" s="37" t="n"/>
+      <c r="C36" s="38" t="n"/>
+      <c r="D36" s="38" t="n"/>
+      <c r="E36" s="38" t="n"/>
+      <c r="F36" s="40" t="n"/>
+      <c r="G36" s="43" t="n"/>
+      <c r="H36" s="43" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="48" t="inlineStr">
-        <is>
-          <t>Código</t>
-        </is>
-      </c>
-      <c r="B37" s="76" t="inlineStr">
-        <is>
-          <t>Descrição</t>
-        </is>
-      </c>
-      <c r="C37" s="58" t="n"/>
-      <c r="D37" s="58" t="n"/>
-      <c r="E37" s="58" t="n"/>
-      <c r="F37" s="58" t="n"/>
-      <c r="G37" s="48" t="inlineStr">
-        <is>
-          <t>Almox Retirada</t>
-        </is>
-      </c>
-      <c r="H37" s="48" t="inlineStr">
-        <is>
-          <t>Qtd</t>
-        </is>
-      </c>
+      <c r="A37" s="43" t="n"/>
+      <c r="B37" s="37" t="n"/>
+      <c r="C37" s="38" t="n"/>
+      <c r="D37" s="38" t="n"/>
+      <c r="E37" s="38" t="n"/>
+      <c r="F37" s="40" t="n"/>
+      <c r="G37" s="43" t="n"/>
+      <c r="H37" s="43" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="43" t="n"/>
@@ -1638,135 +1568,105 @@
       <c r="G42" s="43" t="n"/>
       <c r="H42" s="43" t="n"/>
     </row>
-    <row r="43">
-      <c r="A43" s="43" t="n"/>
-      <c r="B43" s="37" t="n"/>
-      <c r="C43" s="38" t="n"/>
-      <c r="D43" s="38" t="n"/>
-      <c r="E43" s="38" t="n"/>
-      <c r="F43" s="40" t="n"/>
-      <c r="G43" s="43" t="n"/>
-      <c r="H43" s="43" t="n"/>
-    </row>
+    <row r="43"/>
     <row r="44">
-      <c r="A44" s="43" t="n"/>
-      <c r="B44" s="37" t="n"/>
-      <c r="C44" s="38" t="n"/>
-      <c r="D44" s="38" t="n"/>
-      <c r="E44" s="38" t="n"/>
-      <c r="F44" s="40" t="n"/>
-      <c r="G44" s="43" t="n"/>
-      <c r="H44" s="43" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="43" t="n"/>
-      <c r="B45" s="37" t="n"/>
-      <c r="C45" s="38" t="n"/>
-      <c r="D45" s="38" t="n"/>
-      <c r="E45" s="38" t="n"/>
-      <c r="F45" s="40" t="n"/>
-      <c r="G45" s="43" t="n"/>
-      <c r="H45" s="43" t="n"/>
-    </row>
-    <row r="46"/>
+      <c r="A44" s="63" t="inlineStr">
+        <is>
+          <t>4. FINALIZAÇÃO</t>
+        </is>
+      </c>
+      <c r="B44" s="58" t="n"/>
+      <c r="C44" s="58" t="n"/>
+      <c r="D44" s="58" t="n"/>
+      <c r="E44" s="58" t="n"/>
+      <c r="F44" s="58" t="n"/>
+      <c r="G44" s="58" t="n"/>
+      <c r="H44" s="59" t="n"/>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Data:</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="n"/>
+      <c r="D46" s="28" t="n"/>
+      <c r="E46" s="29" t="inlineStr">
+        <is>
+          <t>Hora:</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n"/>
+      <c r="G46" s="30" t="n"/>
+    </row>
     <row r="47">
-      <c r="A47" s="63" t="inlineStr">
-        <is>
-          <t>4. FINALIZAÇÃO</t>
-        </is>
-      </c>
-      <c r="B47" s="58" t="n"/>
-      <c r="C47" s="58" t="n"/>
-      <c r="D47" s="58" t="n"/>
-      <c r="E47" s="58" t="n"/>
-      <c r="F47" s="58" t="n"/>
-      <c r="G47" s="58" t="n"/>
-      <c r="H47" s="59" t="n"/>
-    </row>
-    <row r="48"/>
-    <row r="49">
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>Data:</t>
-        </is>
-      </c>
-      <c r="C49" s="33" t="n"/>
-      <c r="D49" s="28" t="n"/>
-      <c r="E49" s="29" t="inlineStr">
-        <is>
-          <t>Hora:</t>
-        </is>
-      </c>
-      <c r="F49" s="27" t="n"/>
-      <c r="G49" s="30" t="n"/>
-    </row>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Responsável Manutenção:</t>
+        </is>
+      </c>
+      <c r="C47" s="44" t="n"/>
+      <c r="D47" s="27" t="n"/>
+      <c r="E47" s="45" t="n"/>
+      <c r="F47" s="46" t="n"/>
+      <c r="G47" s="47" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>OK Cliente:</t>
+        </is>
+      </c>
+      <c r="C48" s="33" t="n"/>
+      <c r="D48" s="34" t="n"/>
+      <c r="E48" s="34" t="n"/>
+      <c r="F48" s="38" t="n"/>
+      <c r="G48" s="40" t="n"/>
+    </row>
+    <row r="49"/>
     <row r="50">
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Responsável Manutenção:</t>
-        </is>
-      </c>
-      <c r="C50" s="44" t="n"/>
-      <c r="D50" s="27" t="n"/>
-      <c r="E50" s="45" t="n"/>
-      <c r="F50" s="46" t="n"/>
-      <c r="G50" s="47" t="n"/>
+      <c r="A50" s="42" t="inlineStr">
+        <is>
+          <t>OBS DO CLIENTE:</t>
+        </is>
+      </c>
+      <c r="C50" s="41" t="n"/>
+      <c r="D50" s="41" t="n"/>
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="41" t="n"/>
+      <c r="G50" s="41" t="n"/>
+      <c r="H50" s="41" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="32" t="inlineStr">
-        <is>
-          <t>OK Cliente:</t>
-        </is>
-      </c>
-      <c r="C51" s="33" t="n"/>
-      <c r="D51" s="34" t="n"/>
-      <c r="E51" s="34" t="n"/>
-      <c r="F51" s="38" t="n"/>
-      <c r="G51" s="40" t="n"/>
-    </row>
-    <row r="52"/>
+      <c r="A51" s="41" t="n"/>
+      <c r="B51" s="41" t="n"/>
+      <c r="C51" s="41" t="n"/>
+      <c r="D51" s="41" t="n"/>
+      <c r="E51" s="41" t="n"/>
+      <c r="F51" s="41" t="n"/>
+      <c r="G51" s="41" t="n"/>
+      <c r="H51" s="41" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="n"/>
+      <c r="B52" s="41" t="n"/>
+      <c r="C52" s="41" t="n"/>
+      <c r="D52" s="41" t="n"/>
+      <c r="E52" s="41" t="n"/>
+      <c r="F52" s="41" t="n"/>
+      <c r="G52" s="41" t="n"/>
+      <c r="H52" s="41" t="n"/>
+    </row>
     <row r="53">
-      <c r="A53" s="42" t="inlineStr">
-        <is>
-          <t>OBS DO CLIENTE:</t>
-        </is>
-      </c>
+      <c r="A53" s="41" t="n"/>
+      <c r="B53" s="41" t="n"/>
       <c r="C53" s="41" t="n"/>
       <c r="D53" s="41" t="n"/>
       <c r="E53" s="41" t="n"/>
       <c r="F53" s="41" t="n"/>
       <c r="G53" s="41" t="n"/>
       <c r="H53" s="41" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="41" t="n"/>
-      <c r="B54" s="41" t="n"/>
-      <c r="C54" s="41" t="n"/>
-      <c r="D54" s="41" t="n"/>
-      <c r="E54" s="41" t="n"/>
-      <c r="F54" s="41" t="n"/>
-      <c r="G54" s="41" t="n"/>
-      <c r="H54" s="41" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="41" t="n"/>
-      <c r="B55" s="41" t="n"/>
-      <c r="C55" s="41" t="n"/>
-      <c r="D55" s="41" t="n"/>
-      <c r="E55" s="41" t="n"/>
-      <c r="F55" s="41" t="n"/>
-      <c r="G55" s="41" t="n"/>
-      <c r="H55" s="41" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="41" t="n"/>
-      <c r="B56" s="41" t="n"/>
-      <c r="C56" s="41" t="n"/>
-      <c r="D56" s="41" t="n"/>
-      <c r="E56" s="41" t="n"/>
-      <c r="F56" s="41" t="n"/>
-      <c r="G56" s="41" t="n"/>
-      <c r="H56" s="41" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>